<commit_message>
Cattle  slurry lab plan
</commit_message>
<xml_diff>
--- a/Lab-acidification-test-before-lab-field-trails/2025-11-11-Titration-cattle-3rd.xlsx
+++ b/Lab-acidification-test-before-lab-field-trails/2025-11-11-Titration-cattle-3rd.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-acidification-test-before-lab-field-trails\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D38DFCA-39CF-4FFB-9191-B6E094676339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3440259-3B15-4AF5-9BC4-B1399921396E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw data" sheetId="1" r:id="rId1"/>
@@ -163,9 +163,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -183,12 +183,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -221,9 +215,9 @@
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="170" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">

</xml_diff>